<commit_message>
test: update directlookups_invalidcell model to include more data points + skip this model for now
</commit_message>
<xml_diff>
--- a/models/directlookups_invalidcell/data/data.xlsx
+++ b/models/directlookups_invalidcell/data/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/campbell/Projects/CI/sdeverywhere1/models/directlookups_invalidcell/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7334F2D-26B8-404A-86CA-6C405322E652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F8CDB7-C70A-7248-9204-1FC9F7E57B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="1240" windowWidth="34240" windowHeight="20320" xr2:uid="{2A9CE952-2567-B242-8C77-9807BA28D863}"/>
+    <workbookView xWindow="17360" yWindow="640" windowWidth="17040" windowHeight="21520" xr2:uid="{2A9CE952-2567-B242-8C77-9807BA28D863}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>ignored 1</t>
   </si>
@@ -901,10 +901,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C10E3E-9A3B-F340-94CC-13DBE9FAC477}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -918,7 +918,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2000</v>
       </c>
@@ -937,8 +937,17 @@
       <c r="G2">
         <v>2003</v>
       </c>
+      <c r="H2">
+        <v>2004</v>
+      </c>
+      <c r="I2">
+        <v>2005</v>
+      </c>
+      <c r="J2">
+        <v>2006</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>10</v>
       </c>
@@ -960,8 +969,17 @@
       <c r="G3">
         <v>60</v>
       </c>
+      <c r="H3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3">
+        <v>80</v>
+      </c>
+      <c r="J3">
+        <v>90</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>110</v>
       </c>
@@ -979,6 +997,12 @@
       </c>
       <c r="G4">
         <v>160</v>
+      </c>
+      <c r="I4">
+        <v>180</v>
+      </c>
+      <c r="J4">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>